<commit_message>
data: align reviewed Model 2 controls and metadata
</commit_message>
<xml_diff>
--- a/Docs/revisione_profili_model2.xlsx
+++ b/Docs/revisione_profili_model2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="R4815665ee96f4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="R4176218543d84565"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -833,12 +833,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Select Right</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Jump Front</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Jump Tail</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Curving</x:t>
@@ -4307,11 +4301,11 @@
       <x:c r="K42" s="1" t="s">
         <x:v>274</x:v>
       </x:c>
-      <x:c r="L42" s="1" t="s">
-        <x:v>275</x:v>
-      </x:c>
-      <x:c r="M42" s="1" t="s">
-        <x:v>276</x:v>
+      <x:c r="L42" s="1" t="str">
+        <x:v>Jump Tail</x:v>
+      </x:c>
+      <x:c r="M42" s="1" t="str">
+        <x:v>Jump Front</x:v>
       </x:c>
       <x:c r="N42" s="1"/>
       <x:c r="O42" s="1"/>
@@ -4332,44 +4326,44 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X42" s="1" t="s">
-        <x:v>277</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="Y42" s="1"/>
       <x:c r="Z42" s="1" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="AA42" s="1"/>
       <x:c r="AB42" s="1" t="str">
-        <x:v>Curving uses Left Analog X and Slide uses Right Analog X. Curving Axis Mode defaults to Inverted (X+ = 00, X- = FF) and offers Normal; Slide is unchanged.</x:v>
+        <x:v>Curving uses Left Analog X and Slide uses Right Analog X. Curving applies the inverted polarity declared in the metadata (X+ = 00, X- = FF); Slide is unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
       <x:c r="A43" s="1" t="s">
-        <x:v>279</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="B43" s="1" t="s">
-        <x:v>280</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="C43" s="1" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D43" s="1" t="s">
-        <x:v>281</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="E43" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F43" s="1" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="G43" s="1" t="s">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="H43" s="1" t="s">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="G43" s="1" t="s">
+      <x:c r="I43" s="1" t="s">
         <x:v>283</x:v>
-      </x:c>
-      <x:c r="H43" s="1" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="I43" s="1" t="s">
-        <x:v>285</x:v>
       </x:c>
       <x:c r="J43" s="1"/>
       <x:c r="K43" s="1"/>
@@ -4401,10 +4395,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="W43" s="1" t="s">
-        <x:v>286</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="X43" s="1" t="s">
-        <x:v>278</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="Y43" s="1"/>
       <x:c r="Z43" s="1"/>
@@ -4415,28 +4409,28 @@
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
       <x:c r="A44" s="1" t="s">
-        <x:v>287</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="B44" s="1" t="s">
-        <x:v>288</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="C44" s="1" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D44" s="1" t="s">
-        <x:v>289</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="E44" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F44" s="1" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="G44" s="1" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="H44" s="1" t="s">
         <x:v>290</x:v>
-      </x:c>
-      <x:c r="G44" s="1" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="H44" s="1" t="s">
-        <x:v>292</x:v>
       </x:c>
       <x:c r="I44" s="1"/>
       <x:c r="J44" s="1"/>
@@ -4449,7 +4443,7 @@
       <x:c r="Q44" s="1"/>
       <x:c r="R44" s="1"/>
       <x:c r="S44" s="1" t="s">
-        <x:v>293</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="T44" s="1" t="s">
         <x:v>42</x:v>
@@ -4464,23 +4458,23 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X44" s="1" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="Y44" s="1" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="Z44" s="1" t="s">
         <x:v>294</x:v>
-      </x:c>
-      <x:c r="Y44" s="1" t="s">
-        <x:v>295</x:v>
-      </x:c>
-      <x:c r="Z44" s="1" t="s">
-        <x:v>296</x:v>
       </x:c>
       <x:c r="AA44" s="1"/>
       <x:c r="AB44" s="1" t="s">
-        <x:v>297</x:v>
+        <x:v>295</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc84bb1cca6c54119"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138e5811bbca4905"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
core: align runtime with SM2-Emu 0.9.9
</commit_message>
<xml_diff>
--- a/Docs/revisione_profili_model2.xlsx
+++ b/Docs/revisione_profili_model2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="R4176218543d84565"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="Rc378a36b88f74b80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -115,139 +115,139 @@
     <x:t xml:space="preserve">Driving: 4-Speed + VR1 + Handbrake</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Handbrake (Analog)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">4-Speed: Neutral</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Shift Down</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Shift Up</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Brake</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Accelerator</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Service A</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Test A</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Coin</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Steering</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">H-Gate: Left / Right</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">H-Gate: Up / Down</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Model 2 Handbrake is analog on IN2 and mapped to South as Handbrake (Analog).</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Daytona USA</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">daytona</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">model2</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">common, vehicle, steering, accelerator, brake, 4-speed gearbox, VR1-VR4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Driving: 4-Speed + VR4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">VR4 (Green)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">VR1 (Red)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">VR2 (Blue)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">VR3 (Yellow)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Profile and positions match Daytona USA 2 / Power Edition.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Manx TT Superbike - DX/Twin</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">manxtt</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Motorcycle racing</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">common, vehicle, bank, throttle, brake, shift up/down, Start/VR</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Driving: Sequential (Manx TT Superbike)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Start / VR</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Bank</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Model 2-specific profile; bank polarity must be verified.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Motor Raid - Twin</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">motoraid</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Motorcycle combat</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">common, vehicle, bank, throttle, brake, shift up/down, Start/VR, Punch, Kick</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Driving: Sequential (Motor Raid)</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Punch and Kick are additional actions specific to Motor Raid.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Super GT 24h</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">sgt24h</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">model2b</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">common, vehicle, steering, accelerator, brake, shift up/down, View 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Driving: Sequential + VR1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">-</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Driving: Sequential + VR1 (Harley-Davidson)</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">VR1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Handbrake (Analog)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">4-Speed: Neutral</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shift Down</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shift Up</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Brake</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Accelerator</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Service A</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Test A</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Coin</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Steering</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">H-Gate: Left / Right</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">H-Gate: Up / Down</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Model 2 Handbrake is analog on IN2 and mapped to South as Handbrake (Analog).</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Daytona USA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">daytona</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">model2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">common, vehicle, steering, accelerator, brake, 4-speed gearbox, VR1-VR4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Driving: 4-Speed + VR4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">VR4 (Green)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">VR1 (Red)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">VR2 (Blue)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">VR3 (Yellow)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Profile and positions match Daytona USA 2 / Power Edition.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Manx TT Superbike - DX/Twin</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">manxtt</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motorcycle racing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">common, vehicle, bank, throttle, brake, shift up/down, Start/VR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Driving: Sequential (Manx TT Superbike)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Start / VR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bank</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Model 2-specific profile; bank polarity must be verified.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motor Raid - Twin</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">motoraid</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Motorcycle combat</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">common, vehicle, bank, throttle, brake, shift up/down, Start/VR, Punch, Kick</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Driving: Sequential (Motor Raid)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Punch and Kick are additional actions specific to Motor Raid.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Super GT 24h</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">sgt24h</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">model2b</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">common, vehicle, steering, accelerator, brake, shift up/down, View 1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Driving: Sequential + VR1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">-</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Driving: Sequential + VR1 (Harley-Davidson)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Rear Brake</x:t>
@@ -1591,67 +1591,67 @@
       <x:c r="G2" s="1" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="H2" s="1" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="I2" s="1"/>
+      <x:c r="H2" s="1"/>
+      <x:c r="I2" s="1" t="str">
+        <x:v>VR1</x:v>
+      </x:c>
       <x:c r="J2" s="1"/>
       <x:c r="K2" s="1"/>
       <x:c r="L2" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="M2" s="1"/>
       <x:c r="N2" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="O2" s="1"/>
       <x:c r="P2" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q2" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q2" s="1" t="s">
+      <x:c r="R2" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R2" s="1" t="s">
+      <x:c r="S2" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S2" s="1" t="s">
+      <x:c r="T2" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T2" s="1" t="s">
+      <x:c r="U2" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U2" s="1" t="s">
+      <x:c r="V2" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V2" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W2" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X2" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y2" s="1"/>
       <x:c r="Z2" s="1" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA2" s="1" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="AA2" s="1" t="s">
+      <x:c r="AB2" s="1" t="s">
         <x:v>47</x:v>
-      </x:c>
-      <x:c r="AB2" s="1" t="s">
-        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="1" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B3" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="s">
+      <x:c r="C3" s="1" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="C3" s="1" t="s">
-        <x:v>51</x:v>
       </x:c>
       <x:c r="D3" s="1" t="s">
         <x:v>31</x:v>
@@ -1660,88 +1660,88 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F3" s="1" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="G3" s="1" t="s">
+      <x:c r="H3" s="1" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="H3" s="1" t="s">
+      <x:c r="I3" s="1" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="I3" s="1" t="s">
+      <x:c r="J3" s="1" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="J3" s="1" t="s">
+      <x:c r="K3" s="1" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="K3" s="1" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="L3" s="1"/>
       <x:c r="M3" s="1"/>
       <x:c r="N3" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="O3" s="1"/>
       <x:c r="P3" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q3" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q3" s="1" t="s">
+      <x:c r="R3" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R3" s="1" t="s">
+      <x:c r="S3" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S3" s="1" t="s">
+      <x:c r="T3" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T3" s="1" t="s">
+      <x:c r="U3" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U3" s="1" t="s">
+      <x:c r="V3" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V3" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W3" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X3" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y3" s="1"/>
       <x:c r="Z3" s="1" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="AA3" s="1" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="AA3" s="1" t="s">
-        <x:v>47</x:v>
-      </x:c>
       <x:c r="AB3" s="1" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
       <x:c r="A4" s="1" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="s">
         <x:v>59</x:v>
-      </x:c>
-      <x:c r="B4" s="1" t="s">
-        <x:v>60</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F4" s="1" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="G4" s="1" t="s">
-        <x:v>63</x:v>
       </x:c>
       <x:c r="H4" s="1"/>
       <x:c r="I4" s="1"/>
@@ -1752,60 +1752,60 @@
       <x:c r="N4" s="1"/>
       <x:c r="O4" s="1"/>
       <x:c r="P4" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q4" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q4" s="1" t="s">
+      <x:c r="R4" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R4" s="1" t="s">
+      <x:c r="S4" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S4" s="1" t="s">
+      <x:c r="T4" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T4" s="1" t="s">
+      <x:c r="U4" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U4" s="1" t="s">
+      <x:c r="V4" s="1" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="V4" s="1" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="W4" s="1" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="X4" s="1" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="X4" s="1" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="Y4" s="1"/>
       <x:c r="Z4" s="1"/>
       <x:c r="AA4" s="1"/>
       <x:c r="AB4" s="1" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="20" customHeight="1">
       <x:c r="A5" s="1" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="B5" s="1" t="s">
-        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F5" s="1" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="G5" s="1" t="s">
-        <x:v>71</x:v>
       </x:c>
       <x:c r="H5" s="1"/>
       <x:c r="I5" s="1"/>
@@ -1820,48 +1820,48 @@
       <x:c r="N5" s="1"/>
       <x:c r="O5" s="1"/>
       <x:c r="P5" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q5" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q5" s="1" t="s">
+      <x:c r="R5" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R5" s="1" t="s">
+      <x:c r="S5" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S5" s="1" t="s">
+      <x:c r="T5" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T5" s="1" t="s">
+      <x:c r="U5" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U5" s="1" t="s">
+      <x:c r="V5" s="1" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="V5" s="1" t="s">
-        <x:v>44</x:v>
-      </x:c>
       <x:c r="W5" s="1" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="X5" s="1" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="X5" s="1" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="Y5" s="1"/>
       <x:c r="Z5" s="1"/>
       <x:c r="AA5" s="1"/>
       <x:c r="AB5" s="1" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="s">
+      <x:c r="C6" s="1" t="s">
         <x:v>74</x:v>
-      </x:c>
-      <x:c r="C6" s="1" t="s">
-        <x:v>75</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
         <x:v>31</x:v>
@@ -1870,15 +1870,15 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F6" s="1" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="G6" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="H6" s="1" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="I6" s="1"/>
+      <x:c r="H6" s="1"/>
+      <x:c r="I6" s="1" t="str">
+        <x:v>VR1</x:v>
+      </x:c>
       <x:c r="J6" s="1"/>
       <x:c r="K6" s="1"/>
       <x:c r="L6" s="1"/>
@@ -1886,31 +1886,31 @@
       <x:c r="N6" s="1"/>
       <x:c r="O6" s="1"/>
       <x:c r="P6" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q6" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q6" s="1" t="s">
+      <x:c r="R6" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R6" s="1" t="s">
+      <x:c r="S6" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S6" s="1" t="s">
+      <x:c r="T6" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T6" s="1" t="s">
+      <x:c r="U6" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U6" s="1" t="s">
+      <x:c r="V6" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V6" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W6" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X6" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y6" s="1"/>
       <x:c r="Z6" s="1"/>
@@ -1921,28 +1921,28 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="F7" s="1" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="G7" s="1" t="s">
+      <x:c r="H7" s="1" t="s">
         <x:v>79</x:v>
-      </x:c>
-      <x:c r="H7" s="1" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="1"/>
@@ -1956,31 +1956,31 @@
       <x:c r="N7" s="1"/>
       <x:c r="O7" s="1"/>
       <x:c r="P7" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q7" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q7" s="1" t="s">
+      <x:c r="R7" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R7" s="1" t="s">
+      <x:c r="S7" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S7" s="1" t="s">
+      <x:c r="T7" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T7" s="1" t="s">
+      <x:c r="U7" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U7" s="1" t="s">
+      <x:c r="V7" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V7" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W7" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X7" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y7" s="1"/>
       <x:c r="Z7" s="1"/>
@@ -1997,7 +1997,7 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
         <x:v>31</x:v>
@@ -2024,31 +2024,31 @@
       <x:c r="N8" s="1"/>
       <x:c r="O8" s="1"/>
       <x:c r="P8" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q8" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q8" s="1" t="s">
+      <x:c r="R8" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R8" s="1" t="s">
+      <x:c r="S8" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S8" s="1" t="s">
+      <x:c r="T8" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T8" s="1" t="s">
+      <x:c r="U8" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U8" s="1" t="s">
+      <x:c r="V8" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V8" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W8" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X8" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y8" s="1"/>
       <x:c r="Z8" s="1"/>
@@ -2092,31 +2092,31 @@
       <x:c r="N9" s="1"/>
       <x:c r="O9" s="1"/>
       <x:c r="P9" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q9" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q9" s="1" t="s">
+      <x:c r="R9" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R9" s="1" t="s">
+      <x:c r="S9" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S9" s="1" t="s">
+      <x:c r="T9" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T9" s="1" t="s">
+      <x:c r="U9" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U9" s="1" t="s">
+      <x:c r="V9" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V9" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W9" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X9" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y9" s="1"/>
       <x:c r="Z9" s="1"/>
@@ -2160,31 +2160,31 @@
       <x:c r="N10" s="1"/>
       <x:c r="O10" s="1"/>
       <x:c r="P10" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q10" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q10" s="1" t="s">
+      <x:c r="R10" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R10" s="1" t="s">
+      <x:c r="S10" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S10" s="1" t="s">
+      <x:c r="T10" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T10" s="1" t="s">
+      <x:c r="U10" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U10" s="1" t="s">
+      <x:c r="V10" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V10" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W10" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X10" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y10" s="1"/>
       <x:c r="Z10" s="1"/>
@@ -2195,68 +2195,68 @@
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F11" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G11" s="1" t="s">
         <x:v>95</x:v>
       </x:c>
       <x:c r="H11" s="1" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="I11" s="1" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="I11" s="1" t="s">
+      <x:c r="J11" s="1" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="J11" s="1" t="s">
+      <x:c r="K11" s="1" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="K11" s="1" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="L11" s="1"/>
       <x:c r="M11" s="1"/>
       <x:c r="N11" s="1"/>
       <x:c r="O11" s="1"/>
       <x:c r="P11" s="1" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="Q11" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="Q11" s="1" t="s">
+      <x:c r="R11" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="R11" s="1" t="s">
+      <x:c r="S11" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="S11" s="1" t="s">
+      <x:c r="T11" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T11" s="1" t="s">
+      <x:c r="U11" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U11" s="1" t="s">
+      <x:c r="V11" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V11" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W11" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X11" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y11" s="1"/>
       <x:c r="Z11" s="1"/>
@@ -2273,7 +2273,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D12" s="1" t="s">
         <x:v>98</x:v>
@@ -2302,13 +2302,13 @@
       <x:c r="R12" s="1"/>
       <x:c r="S12" s="1"/>
       <x:c r="T12" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U12" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U12" s="1" t="s">
+      <x:c r="V12" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V12" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W12" s="1" t="s">
         <x:v>22</x:v>
@@ -2364,13 +2364,13 @@
       <x:c r="R13" s="1"/>
       <x:c r="S13" s="1"/>
       <x:c r="T13" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U13" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U13" s="1" t="s">
+      <x:c r="V13" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V13" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W13" s="1" t="s">
         <x:v>22</x:v>
@@ -2395,7 +2395,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
         <x:v>98</x:v>
@@ -2424,13 +2424,13 @@
       <x:c r="R14" s="1"/>
       <x:c r="S14" s="1"/>
       <x:c r="T14" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U14" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U14" s="1" t="s">
+      <x:c r="V14" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V14" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W14" s="1" t="s">
         <x:v>22</x:v>
@@ -2455,7 +2455,7 @@
         <x:v>115</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
         <x:v>98</x:v>
@@ -2486,13 +2486,13 @@
       <x:c r="R15" s="1"/>
       <x:c r="S15" s="1"/>
       <x:c r="T15" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U15" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U15" s="1" t="s">
+      <x:c r="V15" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V15" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W15" s="1" t="s">
         <x:v>22</x:v>
@@ -2548,13 +2548,13 @@
       <x:c r="R16" s="1"/>
       <x:c r="S16" s="1"/>
       <x:c r="T16" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U16" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U16" s="1" t="s">
+      <x:c r="V16" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V16" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W16" s="1" t="s">
         <x:v>22</x:v>
@@ -2610,13 +2610,13 @@
       <x:c r="R17" s="1"/>
       <x:c r="S17" s="1"/>
       <x:c r="T17" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U17" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U17" s="1" t="s">
+      <x:c r="V17" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V17" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W17" s="1" t="s">
         <x:v>22</x:v>
@@ -2674,13 +2674,13 @@
       <x:c r="R18" s="1"/>
       <x:c r="S18" s="1"/>
       <x:c r="T18" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U18" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U18" s="1" t="s">
+      <x:c r="V18" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V18" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W18" s="1" t="s">
         <x:v>22</x:v>
@@ -2746,13 +2746,13 @@
       <x:c r="R19" s="1"/>
       <x:c r="S19" s="1"/>
       <x:c r="T19" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U19" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U19" s="1" t="s">
+      <x:c r="V19" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V19" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W19" s="1" t="s">
         <x:v>22</x:v>
@@ -2814,13 +2814,13 @@
       <x:c r="R20" s="1"/>
       <x:c r="S20" s="1"/>
       <x:c r="T20" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U20" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U20" s="1" t="s">
+      <x:c r="V20" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V20" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W20" s="1" t="s">
         <x:v>22</x:v>
@@ -2841,7 +2841,7 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
         <x:v>155</x:v>
@@ -2880,13 +2880,13 @@
       <x:c r="R21" s="1"/>
       <x:c r="S21" s="1"/>
       <x:c r="T21" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U21" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U21" s="1" t="s">
+      <x:c r="V21" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V21" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W21" s="1" t="s">
         <x:v>22</x:v>
@@ -2909,7 +2909,7 @@
         <x:v>159</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
         <x:v>155</x:v>
@@ -2948,13 +2948,13 @@
       <x:c r="R22" s="1"/>
       <x:c r="S22" s="1"/>
       <x:c r="T22" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U22" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U22" s="1" t="s">
+      <x:c r="V22" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V22" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W22" s="1" t="s">
         <x:v>22</x:v>
@@ -3018,13 +3018,13 @@
       <x:c r="R23" s="1"/>
       <x:c r="S23" s="1"/>
       <x:c r="T23" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U23" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U23" s="1" t="s">
+      <x:c r="V23" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V23" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W23" s="1" t="s">
         <x:v>22</x:v>
@@ -3086,13 +3086,13 @@
       <x:c r="R24" s="1"/>
       <x:c r="S24" s="1"/>
       <x:c r="T24" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U24" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U24" s="1" t="s">
+      <x:c r="V24" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V24" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W24" s="1" t="s">
         <x:v>22</x:v>
@@ -3113,7 +3113,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="C25" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D25" s="1" t="s">
         <x:v>171</x:v>
@@ -3154,13 +3154,13 @@
       <x:c r="R25" s="1"/>
       <x:c r="S25" s="1"/>
       <x:c r="T25" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U25" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U25" s="1" t="s">
+      <x:c r="V25" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V25" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W25" s="1" t="s">
         <x:v>22</x:v>
@@ -3181,7 +3181,7 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
         <x:v>171</x:v>
@@ -3222,13 +3222,13 @@
       <x:c r="R26" s="1"/>
       <x:c r="S26" s="1"/>
       <x:c r="T26" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U26" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U26" s="1" t="s">
+      <x:c r="V26" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V26" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W26" s="1" t="s">
         <x:v>22</x:v>
@@ -3290,13 +3290,13 @@
       <x:c r="R27" s="1"/>
       <x:c r="S27" s="1"/>
       <x:c r="T27" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U27" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U27" s="1" t="s">
+      <x:c r="V27" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V27" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W27" s="1" t="s">
         <x:v>22</x:v>
@@ -3317,7 +3317,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="C28" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D28" s="1" t="s">
         <x:v>171</x:v>
@@ -3358,13 +3358,13 @@
       <x:c r="R28" s="1"/>
       <x:c r="S28" s="1"/>
       <x:c r="T28" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U28" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U28" s="1" t="s">
+      <x:c r="V28" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V28" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W28" s="1" t="s">
         <x:v>22</x:v>
@@ -3385,7 +3385,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="C29" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D29" s="1" t="s">
         <x:v>171</x:v>
@@ -3426,13 +3426,13 @@
       <x:c r="R29" s="1"/>
       <x:c r="S29" s="1"/>
       <x:c r="T29" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U29" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U29" s="1" t="s">
+      <x:c r="V29" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V29" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W29" s="1" t="s">
         <x:v>22</x:v>
@@ -3447,22 +3447,22 @@
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G30" s="1" t="s">
         <x:v>190</x:v>
@@ -3496,13 +3496,13 @@
       <x:c r="R30" s="1"/>
       <x:c r="S30" s="1"/>
       <x:c r="T30" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U30" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U30" s="1" t="s">
+      <x:c r="V30" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V30" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W30" s="1" t="s">
         <x:v>22</x:v>
@@ -3523,7 +3523,7 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="C31" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D31" s="1" t="s">
         <x:v>196</x:v>
@@ -3562,13 +3562,13 @@
       <x:c r="R31" s="1"/>
       <x:c r="S31" s="1"/>
       <x:c r="T31" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U31" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U31" s="1" t="s">
+      <x:c r="V31" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V31" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W31" s="1" t="s">
         <x:v>22</x:v>
@@ -3589,7 +3589,7 @@
         <x:v>200</x:v>
       </x:c>
       <x:c r="C32" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D32" s="1" t="s">
         <x:v>196</x:v>
@@ -3628,13 +3628,13 @@
       <x:c r="R32" s="1"/>
       <x:c r="S32" s="1"/>
       <x:c r="T32" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U32" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U32" s="1" t="s">
+      <x:c r="V32" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V32" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W32" s="1" t="s">
         <x:v>22</x:v>
@@ -3694,13 +3694,13 @@
       <x:c r="R33" s="1"/>
       <x:c r="S33" s="1"/>
       <x:c r="T33" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U33" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U33" s="1" t="s">
+      <x:c r="V33" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V33" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W33" s="1" t="s">
         <x:v>22</x:v>
@@ -3721,7 +3721,7 @@
         <x:v>204</x:v>
       </x:c>
       <x:c r="C34" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D34" s="1" t="s">
         <x:v>205</x:v>
@@ -3762,13 +3762,13 @@
       <x:c r="R34" s="1"/>
       <x:c r="S34" s="1"/>
       <x:c r="T34" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U34" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U34" s="1" t="s">
+      <x:c r="V34" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V34" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W34" s="1" t="s">
         <x:v>22</x:v>
@@ -3789,7 +3789,7 @@
         <x:v>212</x:v>
       </x:c>
       <x:c r="C35" s="1" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D35" s="1" t="s">
         <x:v>213</x:v>
@@ -3824,13 +3824,13 @@
         <x:v>219</x:v>
       </x:c>
       <x:c r="T35" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U35" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U35" s="1" t="s">
+      <x:c r="V35" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V35" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W35" s="1" t="s">
         <x:v>22</x:v>
@@ -3859,7 +3859,7 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
         <x:v>227</x:v>
@@ -3901,22 +3901,22 @@
       </x:c>
       <x:c r="R36" s="1"/>
       <x:c r="S36" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="T36" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="T36" s="1" t="s">
+      <x:c r="U36" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U36" s="1" t="s">
+      <x:c r="V36" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V36" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W36" s="1" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="X36" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="Y36" s="1" t="s">
         <x:v>230</x:v>
@@ -3931,22 +3931,22 @@
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
       <x:c r="A37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F37" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G37" s="1" t="s">
         <x:v>231</x:v>
@@ -3972,13 +3972,13 @@
         <x:v>235</x:v>
       </x:c>
       <x:c r="T37" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U37" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U37" s="1" t="s">
+      <x:c r="V37" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V37" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W37" s="1" t="s">
         <x:v>232</x:v>
@@ -4001,22 +4001,22 @@
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
       <x:c r="A38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F38" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G38" s="1" t="s">
         <x:v>240</x:v>
@@ -4036,13 +4036,13 @@
       <x:c r="R38" s="1"/>
       <x:c r="S38" s="1"/>
       <x:c r="T38" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U38" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U38" s="1" t="s">
+      <x:c r="V38" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V38" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W38" s="1" t="s">
         <x:v>22</x:v>
@@ -4059,22 +4059,22 @@
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F39" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G39" s="1" t="s">
         <x:v>243</x:v>
@@ -4102,13 +4102,13 @@
       <x:c r="R39" s="1"/>
       <x:c r="S39" s="1"/>
       <x:c r="T39" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U39" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U39" s="1" t="s">
+      <x:c r="V39" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V39" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W39" s="1" t="s">
         <x:v>244</x:v>
@@ -4174,13 +4174,13 @@
       <x:c r="R40" s="1"/>
       <x:c r="S40" s="1"/>
       <x:c r="T40" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U40" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U40" s="1" t="s">
+      <x:c r="V40" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V40" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W40" s="1" t="s">
         <x:v>22</x:v>
@@ -4199,22 +4199,22 @@
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
       <x:c r="A41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F41" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G41" s="1" t="s">
         <x:v>261</x:v>
@@ -4248,13 +4248,13 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="T41" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U41" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U41" s="1" t="s">
+      <x:c r="V41" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V41" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W41" s="1" t="s">
         <x:v>22</x:v>
@@ -4314,13 +4314,13 @@
       <x:c r="R42" s="1"/>
       <x:c r="S42" s="1"/>
       <x:c r="T42" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U42" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U42" s="1" t="s">
+      <x:c r="V42" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V42" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W42" s="1" t="s">
         <x:v>22</x:v>
@@ -4386,13 +4386,13 @@
       <x:c r="R43" s="1"/>
       <x:c r="S43" s="1"/>
       <x:c r="T43" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U43" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U43" s="1" t="s">
+      <x:c r="V43" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V43" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W43" s="1" t="s">
         <x:v>284</x:v>
@@ -4446,13 +4446,13 @@
         <x:v>291</x:v>
       </x:c>
       <x:c r="T44" s="1" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="U44" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="U44" s="1" t="s">
+      <x:c r="V44" s="1" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="V44" s="1" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="W44" s="1" t="s">
         <x:v>22</x:v>
@@ -4474,7 +4474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138e5811bbca4905"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163a20534d6f4b34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record completed runtime and validation work
</commit_message>
<xml_diff>
--- a/Docs/revisione_profili_model2.xlsx
+++ b/Docs/revisione_profili_model2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="Rc378a36b88f74b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="Rafc34e95452443d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3051,7 +3051,7 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="E24" s="1" t="str">
-        <x:v>2 players</x:v>
+        <x:v>4 players</x:v>
       </x:c>
       <x:c r="F24" s="1" t="s">
         <x:v>167</x:v>
@@ -3102,7 +3102,7 @@
       <x:c r="Z24" s="1"/>
       <x:c r="AA24" s="1"/>
       <x:c r="AB24" s="1" t="str">
-        <x:v>P1/P2 use the current SM2 input path; MAME documents dedicated multiplexing for P3/P4.</x:v>
+        <x:v>P1-P4 use the MAME-documented port-F multiplexed matrix; the input profile is implemented.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
@@ -4474,7 +4474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163a20534d6f4b34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R426d9c7f21014c6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Manx TT and Motor Raid bindings
</commit_message>
<xml_diff>
--- a/Docs/revisione_profili_model2.xlsx
+++ b/Docs/revisione_profili_model2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="Rafc34e95452443d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profili" sheetId="1" r:id="Rf7858a5ba0c8469e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -215,9 +215,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Motorcycle combat</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">common, vehicle, bank, throttle, brake, shift up/down, Start/VR, Punch, Kick</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Driving: Sequential (Motor Raid)</x:t>
@@ -1744,7 +1741,9 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="H4" s="1"/>
-      <x:c r="I4" s="1"/>
+      <x:c r="I4" s="1" t="str">
+        <x:v>Start / VR</x:v>
+      </x:c>
       <x:c r="J4" s="1"/>
       <x:c r="K4" s="1"/>
       <x:c r="L4" s="1"/>
@@ -1801,11 +1800,11 @@
       <x:c r="E5" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="F5" s="1" t="s">
+      <x:c r="F5" s="1" t="str">
+        <x:v>common, vehicle, bank, throttle, brake, Start/VR, Punch, Kick</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="s">
         <x:v>69</x:v>
-      </x:c>
-      <x:c r="G5" s="1" t="s">
-        <x:v>70</x:v>
       </x:c>
       <x:c r="H5" s="1"/>
       <x:c r="I5" s="1"/>
@@ -1819,11 +1818,11 @@
       </x:c>
       <x:c r="N5" s="1"/>
       <x:c r="O5" s="1"/>
-      <x:c r="P5" s="1" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="Q5" s="1" t="s">
-        <x:v>38</x:v>
+      <x:c r="P5" s="1" t="str">
+        <x:v>Kick</x:v>
+      </x:c>
+      <x:c r="Q5" s="1" t="str">
+        <x:v>Punch</x:v>
       </x:c>
       <x:c r="R5" s="1" t="s">
         <x:v>39</x:v>
@@ -1850,18 +1849,18 @@
       <x:c r="Z5" s="1"/>
       <x:c r="AA5" s="1"/>
       <x:c r="AB5" s="1" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="1" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B6" s="1" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="s">
+      <x:c r="C6" s="1" t="s">
         <x:v>73</x:v>
-      </x:c>
-      <x:c r="C6" s="1" t="s">
-        <x:v>74</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
         <x:v>31</x:v>
@@ -1870,10 +1869,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F6" s="1" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="G6" s="1" t="s">
-        <x:v>76</x:v>
       </x:c>
       <x:c r="H6" s="1"/>
       <x:c r="I6" s="1" t="str">
@@ -1921,37 +1920,37 @@
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C7" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="D7" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="E7" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="F7" s="1" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="G7" s="1" t="s">
+      <x:c r="H7" s="1" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="H7" s="1" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="1"/>
       <x:c r="K7" s="1"/>
       <x:c r="L7" s="1" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="M7" s="1" t="s">
         <x:v>80</x:v>
-      </x:c>
-      <x:c r="M7" s="1" t="s">
-        <x:v>81</x:v>
       </x:c>
       <x:c r="N7" s="1"/>
       <x:c r="O7" s="1"/>
@@ -1986,18 +1985,18 @@
       <x:c r="Z7" s="1"/>
       <x:c r="AA7" s="1"/>
       <x:c r="AB7" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="1" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B8" s="1" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B8" s="1" t="s">
-        <x:v>84</x:v>
-      </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
         <x:v>31</x:v>
@@ -2006,16 +2005,16 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F8" s="1" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="G8" s="1" t="s">
+      <x:c r="H8" s="1" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="H8" s="1" t="s">
+      <x:c r="I8" s="1" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="I8" s="1" t="s">
-        <x:v>88</x:v>
       </x:c>
       <x:c r="J8" s="1"/>
       <x:c r="K8" s="1"/>
@@ -2054,18 +2053,18 @@
       <x:c r="Z8" s="1"/>
       <x:c r="AA8" s="1"/>
       <x:c r="AB8" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="1" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
+      <x:c r="C9" s="1" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>92</x:v>
       </x:c>
       <x:c r="D9" s="1" t="s">
         <x:v>31</x:v>
@@ -2074,16 +2073,16 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="s">
+      <x:c r="H9" s="1" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="H9" s="1" t="s">
+      <x:c r="I9" s="1" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="I9" s="1" t="s">
-        <x:v>88</x:v>
       </x:c>
       <x:c r="J9" s="1"/>
       <x:c r="K9" s="1"/>
@@ -2122,18 +2121,18 @@
       <x:c r="Z9" s="1"/>
       <x:c r="AA9" s="1"/>
       <x:c r="AB9" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="1" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>94</x:v>
-      </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>92</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
         <x:v>31</x:v>
@@ -2142,16 +2141,16 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="F10" s="1" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="G10" s="1" t="s">
+      <x:c r="H10" s="1" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="H10" s="1" t="s">
+      <x:c r="I10" s="1" t="s">
         <x:v>87</x:v>
-      </x:c>
-      <x:c r="I10" s="1" t="s">
-        <x:v>88</x:v>
       </x:c>
       <x:c r="J10" s="1"/>
       <x:c r="K10" s="1"/>
@@ -2190,30 +2189,30 @@
       <x:c r="Z10" s="1"/>
       <x:c r="AA10" s="1"/>
       <x:c r="AB10" s="1" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F11" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G11" s="1" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="H11" s="1" t="s">
         <x:v>53</x:v>
@@ -2262,37 +2261,37 @@
       <x:c r="Z11" s="1"/>
       <x:c r="AA11" s="1"/>
       <x:c r="AB11" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="1" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="s">
+      <x:c r="C12" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="s">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="C12" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D12" s="1" t="s">
+      <x:c r="E12" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E12" s="1" t="s">
+      <x:c r="F12" s="1" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="F12" s="1" t="s">
+      <x:c r="G12" s="1" t="s">
         <x:v>100</x:v>
-      </x:c>
-      <x:c r="G12" s="1" t="s">
-        <x:v>101</x:v>
       </x:c>
       <x:c r="H12" s="1"/>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="1"/>
       <x:c r="K12" s="1"/>
       <x:c r="L12" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M12" s="1"/>
       <x:c r="N12" s="1"/>
@@ -2314,48 +2313,48 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X12" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y12" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y12" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z12" s="1"/>
       <x:c r="AA12" s="1"/>
       <x:c r="AB12" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="1" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B13" s="1" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="s">
+      <x:c r="C13" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="C13" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D13" s="1" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="E13" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F13" s="1" t="s">
-        <x:v>108</x:v>
-      </x:c>
       <x:c r="G13" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H13" s="1"/>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
       <x:c r="K13" s="1"/>
       <x:c r="L13" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M13" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="N13" s="1"/>
       <x:c r="O13" s="1"/>
@@ -2376,45 +2375,45 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X13" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y13" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y13" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z13" s="1"/>
       <x:c r="AA13" s="1"/>
       <x:c r="AB13" s="1" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="1" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="B14" s="1" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="s">
-        <x:v>112</x:v>
-      </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D14" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E14" s="1" t="s">
+      <x:c r="F14" s="1" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="F14" s="1" t="s">
+      <x:c r="G14" s="1" t="s">
         <x:v>100</x:v>
-      </x:c>
-      <x:c r="G14" s="1" t="s">
-        <x:v>101</x:v>
       </x:c>
       <x:c r="H14" s="1"/>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
       <x:c r="K14" s="1"/>
       <x:c r="L14" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M14" s="1"/>
       <x:c r="N14" s="1"/>
@@ -2436,48 +2435,48 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X14" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y14" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y14" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z14" s="1"/>
       <x:c r="AA14" s="1"/>
       <x:c r="AB14" s="1" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="1" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="B15" s="1" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="B15" s="1" t="s">
-        <x:v>115</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="D15" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E15" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
       <x:c r="F15" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G15" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H15" s="1"/>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
       <x:c r="K15" s="1"/>
       <x:c r="L15" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M15" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="N15" s="1"/>
       <x:c r="O15" s="1"/>
@@ -2498,48 +2497,48 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X15" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y15" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y15" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z15" s="1"/>
       <x:c r="AA15" s="1"/>
       <x:c r="AB15" s="1" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="1" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="B16" s="1" t="s">
-        <x:v>118</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D16" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E16" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
       <x:c r="F16" s="1" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G16" s="1" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H16" s="1"/>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
       <x:c r="K16" s="1"/>
       <x:c r="L16" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M16" s="1" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="N16" s="1"/>
       <x:c r="O16" s="1"/>
@@ -2560,48 +2559,48 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X16" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y16" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y16" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z16" s="1"/>
       <x:c r="AA16" s="1"/>
       <x:c r="AB16" s="1" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="1" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="s">
+      <x:c r="C17" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E17" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F17" s="1" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="C17" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D17" s="1" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="E17" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F17" s="1" t="s">
+      <x:c r="G17" s="1" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="G17" s="1" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="H17" s="1"/>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
       <x:c r="K17" s="1"/>
       <x:c r="L17" s="1" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="M17" s="1" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="N17" s="1"/>
       <x:c r="O17" s="1"/>
@@ -2622,38 +2621,38 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X17" s="1" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="Y17" s="1" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="Y17" s="1" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="Z17" s="1"/>
       <x:c r="AA17" s="1"/>
       <x:c r="AB17" s="1" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="1" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="B18" s="1" t="s">
         <x:v>125</x:v>
-      </x:c>
-      <x:c r="B18" s="1" t="s">
-        <x:v>126</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D18" s="1" t="s">
-        <x:v>127</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E18" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F18" s="1" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="G18" s="1" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="G18" s="1" t="s">
-        <x:v>129</x:v>
       </x:c>
       <x:c r="H18" s="1" t="str">
         <x:v>View Change</x:v>
@@ -2662,10 +2661,10 @@
       <x:c r="J18" s="1"/>
       <x:c r="K18" s="1"/>
       <x:c r="L18" s="1" t="s">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="M18" s="1" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="N18" s="1"/>
       <x:c r="O18" s="1"/>
@@ -2686,10 +2685,10 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X18" s="1" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="Y18" s="1" t="s">
         <x:v>131</x:v>
-      </x:c>
-      <x:c r="Y18" s="1" t="s">
-        <x:v>132</x:v>
       </x:c>
       <x:c r="Z18" s="1"/>
       <x:c r="AA18" s="1"/>
@@ -2699,46 +2698,46 @@
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="1" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="B19" s="1" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="B19" s="1" t="s">
+      <x:c r="C19" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D19" s="1" t="s">
         <x:v>134</x:v>
-      </x:c>
-      <x:c r="C19" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D19" s="1" t="s">
-        <x:v>135</x:v>
       </x:c>
       <x:c r="E19" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F19" s="1" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="G19" s="1" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="G19" s="1" t="s">
+      <x:c r="H19" s="1" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="H19" s="1" t="s">
+      <x:c r="I19" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I19" s="1" t="s">
+      <x:c r="J19" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J19" s="1" t="s">
+      <x:c r="K19" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K19" s="1" t="s">
+      <x:c r="L19" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L19" s="1" t="s">
+      <x:c r="M19" s="1" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="M19" s="1" t="s">
+      <x:c r="N19" s="1" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="N19" s="1" t="s">
-        <x:v>144</x:v>
       </x:c>
       <x:c r="O19" s="1"/>
       <x:c r="P19" s="1"/>
@@ -2762,42 +2761,42 @@
       <x:c r="Z19" s="1"/>
       <x:c r="AA19" s="1"/>
       <x:c r="AB19" s="1" t="s">
-        <x:v>145</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="1" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="B20" s="1" t="s">
         <x:v>146</x:v>
-      </x:c>
-      <x:c r="B20" s="1" t="s">
-        <x:v>147</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D20" s="1" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F20" s="1" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="E20" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F20" s="1" t="s">
+      <x:c r="G20" s="1" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="G20" s="1" t="s">
-        <x:v>150</x:v>
-      </x:c>
       <x:c r="H20" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I20" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I20" s="1" t="s">
+      <x:c r="J20" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J20" s="1" t="s">
+      <x:c r="K20" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K20" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L20" s="1" t="str">
         <x:v>Kick</x:v>
@@ -2806,7 +2805,7 @@
         <x:v>Punch</x:v>
       </x:c>
       <x:c r="N20" s="1" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="O20" s="1"/>
       <x:c r="P20" s="1"/>
@@ -2830,48 +2829,48 @@
       <x:c r="Z20" s="1"/>
       <x:c r="AA20" s="1"/>
       <x:c r="AB20" s="1" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="1" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="B21" s="1" t="s">
         <x:v>153</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="s">
+      <x:c r="C21" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D21" s="1" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="C21" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D21" s="1" t="s">
+      <x:c r="E21" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F21" s="1" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="E21" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F21" s="1" t="s">
+      <x:c r="G21" s="1" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="G21" s="1" t="s">
-        <x:v>157</x:v>
-      </x:c>
       <x:c r="H21" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I21" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I21" s="1" t="s">
+      <x:c r="J21" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J21" s="1" t="s">
+      <x:c r="K21" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K21" s="1" t="s">
+      <x:c r="L21" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L21" s="1" t="s">
+      <x:c r="M21" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="M21" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="N21" s="1"/>
       <x:c r="O21" s="1"/>
@@ -2903,43 +2902,43 @@
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
       <x:c r="A22" s="1" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="B22" s="1" t="s">
-        <x:v>159</x:v>
-      </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D22" s="1" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="E22" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F22" s="1" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="E22" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F22" s="1" t="s">
+      <x:c r="G22" s="1" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="G22" s="1" t="s">
-        <x:v>157</x:v>
-      </x:c>
       <x:c r="H22" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I22" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I22" s="1" t="s">
+      <x:c r="J22" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J22" s="1" t="s">
+      <x:c r="K22" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K22" s="1" t="s">
+      <x:c r="L22" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L22" s="1" t="s">
+      <x:c r="M22" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="M22" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="N22" s="1"/>
       <x:c r="O22" s="1"/>
@@ -2971,46 +2970,46 @@
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
       <x:c r="A23" s="1" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="B23" s="1" t="s">
         <x:v>160</x:v>
-      </x:c>
-      <x:c r="B23" s="1" t="s">
-        <x:v>161</x:v>
       </x:c>
       <x:c r="C23" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D23" s="1" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="E23" s="1" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="F23" s="1" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="G23" s="1" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="H23" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I23" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I23" s="1" t="s">
+      <x:c r="J23" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J23" s="1" t="s">
+      <x:c r="K23" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K23" s="1" t="s">
+      <x:c r="L23" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L23" s="1" t="s">
+      <x:c r="M23" s="1" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="M23" s="1" t="s">
+      <x:c r="N23" s="1" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="N23" s="1" t="s">
-        <x:v>144</x:v>
       </x:c>
       <x:c r="O23" s="1"/>
       <x:c r="P23" s="1"/>
@@ -3034,51 +3033,51 @@
       <x:c r="Z23" s="1"/>
       <x:c r="AA23" s="1"/>
       <x:c r="AB23" s="1" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
       <x:c r="A24" s="1" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B24" s="1" t="s">
         <x:v>164</x:v>
-      </x:c>
-      <x:c r="B24" s="1" t="s">
-        <x:v>165</x:v>
       </x:c>
       <x:c r="C24" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D24" s="1" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E24" s="1" t="str">
         <x:v>4 players</x:v>
       </x:c>
       <x:c r="F24" s="1" t="s">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="G24" s="1" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="G24" s="1" t="s">
-        <x:v>168</x:v>
-      </x:c>
       <x:c r="H24" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I24" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I24" s="1" t="s">
+      <x:c r="J24" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J24" s="1" t="s">
+      <x:c r="K24" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K24" s="1" t="s">
+      <x:c r="L24" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L24" s="1" t="s">
+      <x:c r="M24" s="1" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="M24" s="1" t="s">
+      <x:c r="N24" s="1" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="N24" s="1" t="s">
-        <x:v>144</x:v>
       </x:c>
       <x:c r="O24" s="1"/>
       <x:c r="P24" s="1"/>
@@ -3107,37 +3106,37 @@
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
       <x:c r="A25" s="1" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B25" s="1" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="B25" s="1" t="s">
+      <x:c r="C25" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="C25" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D25" s="1" t="s">
+      <x:c r="E25" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F25" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G25" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="E25" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F25" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G25" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="H25" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I25" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I25" s="1" t="s">
+      <x:c r="J25" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J25" s="1" t="s">
+      <x:c r="K25" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K25" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L25" s="1" t="str">
         <x:v>Kick</x:v>
@@ -3146,7 +3145,7 @@
         <x:v>Punch</x:v>
       </x:c>
       <x:c r="N25" s="1" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="O25" s="1"/>
       <x:c r="P25" s="1"/>
@@ -3170,42 +3169,42 @@
       <x:c r="Z25" s="1"/>
       <x:c r="AA25" s="1"/>
       <x:c r="AB25" s="1" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
       <x:c r="A26" s="1" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="B26" s="1" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="B26" s="1" t="s">
-        <x:v>176</x:v>
-      </x:c>
       <x:c r="C26" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D26" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E26" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F26" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G26" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="E26" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F26" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G26" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="H26" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I26" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I26" s="1" t="s">
+      <x:c r="J26" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J26" s="1" t="s">
+      <x:c r="K26" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K26" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L26" s="1" t="str">
         <x:v>Kick</x:v>
@@ -3214,7 +3213,7 @@
         <x:v>Punch</x:v>
       </x:c>
       <x:c r="N26" s="1" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="O26" s="1"/>
       <x:c r="P26" s="1"/>
@@ -3238,42 +3237,42 @@
       <x:c r="Z26" s="1"/>
       <x:c r="AA26" s="1"/>
       <x:c r="AB26" s="1" t="s">
-        <x:v>177</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
       <x:c r="A27" s="1" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B27" s="1" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="B27" s="1" t="s">
-        <x:v>179</x:v>
       </x:c>
       <x:c r="C27" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D27" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E27" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F27" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G27" s="1" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="E27" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F27" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G27" s="1" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="H27" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I27" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I27" s="1" t="s">
+      <x:c r="J27" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J27" s="1" t="s">
+      <x:c r="K27" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K27" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L27" s="1" t="str">
         <x:v>Kick</x:v>
@@ -3282,7 +3281,7 @@
         <x:v>Punch</x:v>
       </x:c>
       <x:c r="N27" s="1" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="O27" s="1"/>
       <x:c r="P27" s="1"/>
@@ -3306,42 +3305,42 @@
       <x:c r="Z27" s="1"/>
       <x:c r="AA27" s="1"/>
       <x:c r="AB27" s="1" t="s">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
       <x:c r="A28" s="1" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B28" s="1" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="B28" s="1" t="s">
+      <x:c r="C28" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D28" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E28" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F28" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G28" s="1" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="C28" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D28" s="1" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="E28" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F28" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G28" s="1" t="s">
-        <x:v>183</x:v>
-      </x:c>
       <x:c r="H28" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I28" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I28" s="1" t="s">
+      <x:c r="J28" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J28" s="1" t="s">
+      <x:c r="K28" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K28" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L28" s="1" t="str">
         <x:v>Kick</x:v>
@@ -3374,42 +3373,42 @@
       <x:c r="Z28" s="1"/>
       <x:c r="AA28" s="1"/>
       <x:c r="AB28" s="1" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
       <x:c r="A29" s="1" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="B29" s="1" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="B29" s="1" t="s">
+      <x:c r="C29" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D29" s="1" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E29" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F29" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G29" s="1" t="s">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="C29" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D29" s="1" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="E29" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F29" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G29" s="1" t="s">
-        <x:v>187</x:v>
-      </x:c>
       <x:c r="H29" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I29" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I29" s="1" t="s">
+      <x:c r="J29" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J29" s="1" t="s">
+      <x:c r="K29" s="1" t="s">
         <x:v>140</x:v>
-      </x:c>
-      <x:c r="K29" s="1" t="s">
-        <x:v>141</x:v>
       </x:c>
       <x:c r="L29" s="1" t="str">
         <x:v>Kick</x:v>
@@ -3418,7 +3417,7 @@
         <x:v>Punch</x:v>
       </x:c>
       <x:c r="N29" s="1" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="O29" s="1"/>
       <x:c r="P29" s="1"/>
@@ -3442,54 +3441,54 @@
       <x:c r="Z29" s="1"/>
       <x:c r="AA29" s="1"/>
       <x:c r="AB29" s="1" t="s">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F30" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G30" s="1" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="H30" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I30" s="1" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J30" s="1" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="K30" s="1" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="L30" s="1" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="H30" s="1" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="I30" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="J30" s="1" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="K30" s="1" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="L30" s="1" t="s">
+      <x:c r="M30" s="1" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="M30" s="1" t="s">
+      <x:c r="N30" s="1" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="N30" s="1" t="s">
-        <x:v>193</x:v>
-      </x:c>
       <x:c r="O30" s="1" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="P30" s="1"/>
       <x:c r="Q30" s="1"/>
@@ -3512,48 +3511,48 @@
       <x:c r="Z30" s="1"/>
       <x:c r="AA30" s="1"/>
       <x:c r="AB30" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
       <x:c r="A31" s="1" t="s">
+        <x:v>193</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="B31" s="1" t="s">
+      <x:c r="C31" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D31" s="1" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="C31" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D31" s="1" t="s">
+      <x:c r="E31" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F31" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G31" s="1" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="E31" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F31" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G31" s="1" t="s">
-        <x:v>197</x:v>
-      </x:c>
       <x:c r="H31" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I31" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I31" s="1" t="s">
+      <x:c r="J31" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J31" s="1" t="s">
+      <x:c r="K31" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K31" s="1" t="s">
+      <x:c r="L31" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L31" s="1" t="s">
+      <x:c r="M31" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="M31" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="N31" s="1"/>
       <x:c r="O31" s="1"/>
@@ -3578,48 +3577,48 @@
       <x:c r="Z31" s="1"/>
       <x:c r="AA31" s="1"/>
       <x:c r="AB31" s="1" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="1" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B32" s="1" t="s">
         <x:v>199</x:v>
       </x:c>
-      <x:c r="B32" s="1" t="s">
-        <x:v>200</x:v>
-      </x:c>
       <x:c r="C32" s="1" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D32" s="1" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="E32" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F32" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G32" s="1" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="E32" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F32" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G32" s="1" t="s">
-        <x:v>197</x:v>
-      </x:c>
       <x:c r="H32" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I32" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I32" s="1" t="s">
+      <x:c r="J32" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J32" s="1" t="s">
+      <x:c r="K32" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K32" s="1" t="s">
+      <x:c r="L32" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L32" s="1" t="s">
+      <x:c r="M32" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="M32" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="N32" s="1"/>
       <x:c r="O32" s="1"/>
@@ -3644,48 +3643,48 @@
       <x:c r="Z32" s="1"/>
       <x:c r="AA32" s="1"/>
       <x:c r="AB32" s="1" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
       <x:c r="A33" s="1" t="s">
-        <x:v>199</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B33" s="1" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C33" s="1" t="s">
         <x:v>30</x:v>
       </x:c>
       <x:c r="D33" s="1" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="E33" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F33" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G33" s="1" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="E33" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F33" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G33" s="1" t="s">
-        <x:v>197</x:v>
-      </x:c>
       <x:c r="H33" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I33" s="1" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I33" s="1" t="s">
+      <x:c r="J33" s="1" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="J33" s="1" t="s">
+      <x:c r="K33" s="1" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="K33" s="1" t="s">
+      <x:c r="L33" s="1" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="L33" s="1" t="s">
+      <x:c r="M33" s="1" t="s">
         <x:v>142</x:v>
-      </x:c>
-      <x:c r="M33" s="1" t="s">
-        <x:v>143</x:v>
       </x:c>
       <x:c r="N33" s="1"/>
       <x:c r="O33" s="1"/>
@@ -3710,51 +3709,51 @@
       <x:c r="Z33" s="1"/>
       <x:c r="AA33" s="1"/>
       <x:c r="AB33" s="1" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
       <x:c r="A34" s="1" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="B34" s="1" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="B34" s="1" t="s">
+      <x:c r="C34" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D34" s="1" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="C34" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D34" s="1" t="s">
+      <x:c r="E34" s="1" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F34" s="1" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="G34" s="1" t="s">
         <x:v>205</x:v>
       </x:c>
-      <x:c r="E34" s="1" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="F34" s="1" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="G34" s="1" t="s">
+      <x:c r="H34" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="I34" s="1" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="J34" s="1" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="K34" s="1" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="L34" s="1" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="H34" s="1" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="I34" s="1" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="J34" s="1" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="K34" s="1" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="L34" s="1" t="s">
+      <x:c r="M34" s="1" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="M34" s="1" t="s">
+      <x:c r="N34" s="1" t="s">
         <x:v>208</x:v>
-      </x:c>
-      <x:c r="N34" s="1" t="s">
-        <x:v>209</x:v>
       </x:c>
       <x:c r="O34" s="1"/>
       <x:c r="P34" s="1"/>
@@ -3778,30 +3777,30 @@
       <x:c r="Z34" s="1"/>
       <x:c r="AA34" s="1"/>
       <x:c r="AB34" s="1" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
       <x:c r="A35" s="1" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="B35" s="1" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="B35" s="1" t="s">
+      <x:c r="C35" s="1" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D35" s="1" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="C35" s="1" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="D35" s="1" t="s">
-        <x:v>213</x:v>
       </x:c>
       <x:c r="E35" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F35" s="1" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="G35" s="1" t="s">
         <x:v>214</x:v>
-      </x:c>
-      <x:c r="G35" s="1" t="s">
-        <x:v>215</x:v>
       </x:c>
       <x:c r="H35" s="1"/>
       <x:c r="I35" s="1"/>
@@ -3812,16 +3811,16 @@
       <x:c r="N35" s="1"/>
       <x:c r="O35" s="1"/>
       <x:c r="P35" s="1" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="Q35" s="1" t="s">
         <x:v>216</x:v>
       </x:c>
-      <x:c r="Q35" s="1" t="s">
+      <x:c r="R35" s="1" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="R35" s="1" t="s">
+      <x:c r="S35" s="1" t="s">
         <x:v>218</x:v>
-      </x:c>
-      <x:c r="S35" s="1" t="s">
-        <x:v>219</x:v>
       </x:c>
       <x:c r="T35" s="1" t="s">
         <x:v>41</x:v>
@@ -3836,39 +3835,39 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X35" s="1" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="Y35" s="1" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="Y35" s="1" t="s">
+      <x:c r="Z35" s="1" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="Z35" s="1" t="s">
+      <x:c r="AA35" s="1" t="s">
         <x:v>222</x:v>
       </x:c>
-      <x:c r="AA35" s="1" t="s">
+      <x:c r="AB35" s="1" t="s">
         <x:v>223</x:v>
-      </x:c>
-      <x:c r="AB35" s="1" t="s">
-        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
       <x:c r="A36" s="1" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="B36" s="1" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="B36" s="1" t="s">
-        <x:v>226</x:v>
       </x:c>
       <x:c r="C36" s="1" t="s">
         <x:v>50</x:v>
       </x:c>
       <x:c r="D36" s="1" t="s">
-        <x:v>227</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="E36" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F36" s="1" t="s">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="G36" s="1" t="str">
         <x:v>Joystick (Analog): Desert Tank + VR3</x:v>
@@ -3884,20 +3883,20 @@
       </x:c>
       <x:c r="K36" s="1"/>
       <x:c r="L36" s="1" t="s">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="M36" s="1" t="s">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="N36" s="1" t="s">
-        <x:v>191</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="O36" s="1"/>
       <x:c r="P36" s="1" t="s">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="Q36" s="1" t="s">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="R36" s="1"/>
       <x:c r="S36" s="1" t="s">
@@ -3919,7 +3918,7 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="Y36" s="1" t="s">
-        <x:v>230</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="Z36" s="1"/>
       <x:c r="AA36" s="1" t="str">
@@ -3931,45 +3930,45 @@
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
       <x:c r="A37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F37" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G37" s="1" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="H37" s="1"/>
       <x:c r="I37" s="1"/>
       <x:c r="J37" s="1"/>
       <x:c r="K37" s="1"/>
       <x:c r="L37" s="1" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="M37" s="1" t="s">
         <x:v>232</x:v>
-      </x:c>
-      <x:c r="M37" s="1" t="s">
-        <x:v>233</x:v>
       </x:c>
       <x:c r="N37" s="1"/>
       <x:c r="O37" s="1"/>
       <x:c r="P37" s="1"/>
       <x:c r="Q37" s="1"/>
       <x:c r="R37" s="1" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="S37" s="1" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="S37" s="1" t="s">
-        <x:v>235</x:v>
       </x:c>
       <x:c r="T37" s="1" t="s">
         <x:v>41</x:v>
@@ -3981,52 +3980,52 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="W37" s="1" t="s">
-        <x:v>232</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="X37" s="1" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="Y37" s="1" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="Y37" s="1" t="s">
+      <x:c r="Z37" s="1" t="s">
         <x:v>237</x:v>
       </x:c>
-      <x:c r="Z37" s="1" t="s">
+      <x:c r="AA37" s="1" t="s">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="AA37" s="1" t="s">
-        <x:v>239</x:v>
-      </x:c>
       <x:c r="AB37" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
       <x:c r="A38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F38" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G38" s="1" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="H38" s="1"/>
       <x:c r="I38" s="1"/>
       <x:c r="J38" s="1"/>
       <x:c r="K38" s="1"/>
       <x:c r="L38" s="1" t="s">
-        <x:v>241</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="M38" s="1"/>
       <x:c r="N38" s="1"/>
@@ -4049,55 +4048,55 @@
       </x:c>
       <x:c r="X38" s="1"/>
       <x:c r="Y38" s="1" t="s">
-        <x:v>242</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="Z38" s="1"/>
       <x:c r="AA38" s="1"/>
       <x:c r="AB38" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F39" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G39" s="1" t="s">
-        <x:v>243</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="H39" s="1"/>
       <x:c r="I39" s="1"/>
       <x:c r="J39" s="1"/>
       <x:c r="K39" s="1"/>
       <x:c r="L39" s="1" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="M39" s="1" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="M39" s="1" t="s">
+      <x:c r="N39" s="1" t="s">
         <x:v>245</x:v>
-      </x:c>
-      <x:c r="N39" s="1" t="s">
-        <x:v>246</x:v>
       </x:c>
       <x:c r="O39" s="1"/>
       <x:c r="P39" s="1" t="s">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c r="Q39" s="1" t="s">
         <x:v>247</x:v>
-      </x:c>
-      <x:c r="Q39" s="1" t="s">
-        <x:v>248</x:v>
       </x:c>
       <x:c r="R39" s="1"/>
       <x:c r="S39" s="1"/>
@@ -4111,58 +4110,58 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="W39" s="1" t="s">
-        <x:v>244</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="X39" s="1" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="Y39" s="1" t="s">
         <x:v>249</x:v>
-      </x:c>
-      <x:c r="Y39" s="1" t="s">
-        <x:v>250</x:v>
       </x:c>
       <x:c r="Z39" s="1"/>
       <x:c r="AA39" s="1"/>
       <x:c r="AB39" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
       <x:c r="A40" s="1" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="B40" s="1" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="B40" s="1" t="s">
+      <x:c r="C40" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D40" s="1" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="C40" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D40" s="1" t="s">
-        <x:v>253</x:v>
       </x:c>
       <x:c r="E40" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F40" s="1" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="G40" s="1" t="s">
         <x:v>254</x:v>
       </x:c>
-      <x:c r="G40" s="1" t="s">
+      <x:c r="H40" s="1" t="s">
         <x:v>255</x:v>
       </x:c>
-      <x:c r="H40" s="1" t="s">
+      <x:c r="I40" s="1" t="s">
         <x:v>256</x:v>
-      </x:c>
-      <x:c r="I40" s="1" t="s">
-        <x:v>257</x:v>
       </x:c>
       <x:c r="J40" s="1"/>
       <x:c r="K40" s="1"/>
       <x:c r="L40" s="1" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="M40" s="1" t="s">
         <x:v>258</x:v>
       </x:c>
-      <x:c r="M40" s="1" t="s">
+      <x:c r="N40" s="1" t="s">
         <x:v>259</x:v>
-      </x:c>
-      <x:c r="N40" s="1" t="s">
-        <x:v>260</x:v>
       </x:c>
       <x:c r="O40" s="1"/>
       <x:c r="P40" s="1" t="str">
@@ -4199,53 +4198,53 @@
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
       <x:c r="A41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F41" s="1" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G41" s="1" t="s">
-        <x:v>261</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="H41" s="1"/>
       <x:c r="I41" s="1"/>
       <x:c r="J41" s="1"/>
       <x:c r="K41" s="1"/>
       <x:c r="L41" s="1" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="M41" s="1" t="s">
         <x:v>262</x:v>
       </x:c>
-      <x:c r="M41" s="1" t="s">
+      <x:c r="N41" s="1" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="N41" s="1" t="s">
+      <x:c r="O41" s="1" t="s">
         <x:v>264</x:v>
       </x:c>
-      <x:c r="O41" s="1" t="s">
-        <x:v>265</x:v>
-      </x:c>
       <x:c r="P41" s="1" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="Q41" s="1" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="R41" s="1" t="s">
         <x:v>262</x:v>
       </x:c>
-      <x:c r="Q41" s="1" t="s">
+      <x:c r="S41" s="1" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="R41" s="1" t="s">
-        <x:v>263</x:v>
-      </x:c>
-      <x:c r="S41" s="1" t="s">
-        <x:v>265</x:v>
       </x:c>
       <x:c r="T41" s="1" t="s">
         <x:v>41</x:v>
@@ -4260,46 +4259,46 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X41" s="1" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="Y41" s="1" t="s">
         <x:v>266</x:v>
-      </x:c>
-      <x:c r="Y41" s="1" t="s">
-        <x:v>267</x:v>
       </x:c>
       <x:c r="Z41" s="1"/>
       <x:c r="AA41" s="1"/>
       <x:c r="AB41" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="20" customHeight="1">
       <x:c r="A42" s="1" t="s">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="B42" s="1" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="B42" s="1" t="s">
+      <x:c r="C42" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D42" s="1" t="s">
         <x:v>269</x:v>
-      </x:c>
-      <x:c r="C42" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D42" s="1" t="s">
-        <x:v>270</x:v>
       </x:c>
       <x:c r="E42" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F42" s="1" t="s">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="G42" s="1" t="s">
         <x:v>271</x:v>
-      </x:c>
-      <x:c r="G42" s="1" t="s">
-        <x:v>272</x:v>
       </x:c>
       <x:c r="H42" s="1"/>
       <x:c r="I42" s="1"/>
       <x:c r="J42" s="1" t="s">
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="K42" s="1" t="s">
         <x:v>273</x:v>
-      </x:c>
-      <x:c r="K42" s="1" t="s">
-        <x:v>274</x:v>
       </x:c>
       <x:c r="L42" s="1" t="str">
         <x:v>Jump Tail</x:v>
@@ -4326,11 +4325,11 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X42" s="1" t="s">
-        <x:v>275</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="Y42" s="1"/>
       <x:c r="Z42" s="1" t="s">
-        <x:v>276</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="AA42" s="1"/>
       <x:c r="AB42" s="1" t="str">
@@ -4339,31 +4338,31 @@
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
       <x:c r="A43" s="1" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="B43" s="1" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="B43" s="1" t="s">
+      <x:c r="C43" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D43" s="1" t="s">
         <x:v>278</x:v>
-      </x:c>
-      <x:c r="C43" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D43" s="1" t="s">
-        <x:v>279</x:v>
       </x:c>
       <x:c r="E43" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F43" s="1" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="G43" s="1" t="s">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="G43" s="1" t="s">
+      <x:c r="H43" s="1" t="s">
         <x:v>281</x:v>
       </x:c>
-      <x:c r="H43" s="1" t="s">
+      <x:c r="I43" s="1" t="s">
         <x:v>282</x:v>
-      </x:c>
-      <x:c r="I43" s="1" t="s">
-        <x:v>283</x:v>
       </x:c>
       <x:c r="J43" s="1"/>
       <x:c r="K43" s="1"/>
@@ -4395,10 +4394,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="W43" s="1" t="s">
-        <x:v>284</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="X43" s="1" t="s">
-        <x:v>276</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="Y43" s="1"/>
       <x:c r="Z43" s="1"/>
@@ -4409,28 +4408,28 @@
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
       <x:c r="A44" s="1" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="B44" s="1" t="s">
         <x:v>285</x:v>
       </x:c>
-      <x:c r="B44" s="1" t="s">
+      <x:c r="C44" s="1" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D44" s="1" t="s">
         <x:v>286</x:v>
-      </x:c>
-      <x:c r="C44" s="1" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D44" s="1" t="s">
-        <x:v>287</x:v>
       </x:c>
       <x:c r="E44" s="1" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="F44" s="1" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="G44" s="1" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="G44" s="1" t="s">
+      <x:c r="H44" s="1" t="s">
         <x:v>289</x:v>
-      </x:c>
-      <x:c r="H44" s="1" t="s">
-        <x:v>290</x:v>
       </x:c>
       <x:c r="I44" s="1"/>
       <x:c r="J44" s="1"/>
@@ -4443,7 +4442,7 @@
       <x:c r="Q44" s="1"/>
       <x:c r="R44" s="1"/>
       <x:c r="S44" s="1" t="s">
-        <x:v>291</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="T44" s="1" t="s">
         <x:v>41</x:v>
@@ -4458,23 +4457,23 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="X44" s="1" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="Y44" s="1" t="s">
         <x:v>292</x:v>
       </x:c>
-      <x:c r="Y44" s="1" t="s">
+      <x:c r="Z44" s="1" t="s">
         <x:v>293</x:v>
-      </x:c>
-      <x:c r="Z44" s="1" t="s">
-        <x:v>294</x:v>
       </x:c>
       <x:c r="AA44" s="1"/>
       <x:c r="AB44" s="1" t="s">
-        <x:v>295</x:v>
+        <x:v>294</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R426d9c7f21014c6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R754fcbe4a92d41c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>